<commit_message>
Final project cleanup and multiple file updates
</commit_message>
<xml_diff>
--- a/data/Finance_Dataset_Dirty.xlsx
+++ b/data/Finance_Dataset_Dirty.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vamsi\DataWarehousingAssignment\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\D\Ellicium\DW assignment - Loparex\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9765757D-F47F-4CAD-BD1D-EDFFF2E89B97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDB5D942-8DB0-4B4B-9209-AAF454819B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="59">
   <si>
     <t>EmployeeID</t>
   </si>
@@ -28,49 +28,175 @@
     <t>ExpenseType</t>
   </si>
   <si>
+    <t>ExpenseAmount</t>
+  </si>
+  <si>
     <t>ExpenseDate</t>
   </si>
   <si>
-    <t>travel</t>
+    <t>ApprovedBy</t>
+  </si>
+  <si>
+    <t>Meals</t>
+  </si>
+  <si>
+    <t>Supplies</t>
+  </si>
+  <si>
+    <t>Travell</t>
   </si>
   <si>
     <t>Travel</t>
   </si>
   <si>
-    <t>MEAL</t>
+    <t>Training</t>
+  </si>
+  <si>
+    <t>Equipment</t>
+  </si>
+  <si>
+    <t>2023-05-21</t>
+  </si>
+  <si>
+    <t>2023-08-13</t>
+  </si>
+  <si>
+    <t>2023-02-19</t>
+  </si>
+  <si>
+    <t>2025-12-31</t>
+  </si>
+  <si>
+    <t>2023-02-03</t>
+  </si>
+  <si>
+    <t>2023-05-01</t>
+  </si>
+  <si>
+    <t>2023-05-31</t>
+  </si>
+  <si>
+    <t>2023-08-02</t>
+  </si>
+  <si>
+    <t>2023-03-14</t>
+  </si>
+  <si>
+    <t>2023-01-12</t>
+  </si>
+  <si>
+    <t>2023-04-30</t>
+  </si>
+  <si>
+    <t>2023-08-08</t>
+  </si>
+  <si>
+    <t>2023-12-08</t>
+  </si>
+  <si>
+    <t>2023-03-02</t>
+  </si>
+  <si>
+    <t>2023-08-07</t>
+  </si>
+  <si>
+    <t>2023-06-17</t>
+  </si>
+  <si>
+    <t>2023-05-30</t>
+  </si>
+  <si>
+    <t>2023-11-20</t>
+  </si>
+  <si>
+    <t>2023-04-12</t>
+  </si>
+  <si>
+    <t>2023-11-12</t>
+  </si>
+  <si>
+    <t>2023-11-13</t>
+  </si>
+  <si>
+    <t>2023-01-13</t>
+  </si>
+  <si>
+    <t>2023-08-24</t>
+  </si>
+  <si>
+    <t>2023-01-30</t>
+  </si>
+  <si>
+    <t>2023-06-24</t>
+  </si>
+  <si>
+    <t>2023-07-27</t>
+  </si>
+  <si>
+    <t>2023-03-24</t>
+  </si>
+  <si>
+    <t>2023-11-28</t>
+  </si>
+  <si>
+    <t>2023-03-31</t>
+  </si>
+  <si>
+    <t>2023-05-07</t>
+  </si>
+  <si>
+    <t>2023-12-04</t>
+  </si>
+  <si>
+    <t>2023-10-14</t>
+  </si>
+  <si>
+    <t>2023-02-18</t>
+  </si>
+  <si>
+    <t>2023-05-26</t>
+  </si>
+  <si>
+    <t>2023-12-01</t>
+  </si>
+  <si>
+    <t>2023-12-07</t>
+  </si>
+  <si>
+    <t>2023-04-27</t>
+  </si>
+  <si>
+    <t>2023-06-19</t>
+  </si>
+  <si>
+    <t>2023-11-19</t>
+  </si>
+  <si>
+    <t>2023-08-30</t>
+  </si>
+  <si>
+    <t>2023-12-20</t>
+  </si>
+  <si>
+    <t>2023-09-18</t>
+  </si>
+  <si>
+    <t>2023-07-31</t>
   </si>
   <si>
     <t>2023-01-10</t>
   </si>
   <si>
-    <t>2023/01/11</t>
-  </si>
-  <si>
-    <t>01-12-2023</t>
-  </si>
-  <si>
-    <t>2023-01-13</t>
-  </si>
-  <si>
-    <t>2023-01-11</t>
-  </si>
-  <si>
-    <t>John Smith</t>
-  </si>
-  <si>
-    <t>john smith</t>
-  </si>
-  <si>
-    <t>Jane Doe</t>
-  </si>
-  <si>
-    <t>Jane DOE</t>
-  </si>
-  <si>
-    <t>ApprovedBy</t>
-  </si>
-  <si>
-    <t>ExpenseAmount</t>
+    <t>2023-11-18</t>
+  </si>
+  <si>
+    <t>2023-10-19</t>
+  </si>
+  <si>
+    <t>2023-04-07</t>
+  </si>
+  <si>
+    <t>2023-03-29</t>
   </si>
 </sst>
 </file>
@@ -438,8 +564,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -452,92 +585,857 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2">
-        <v>101</v>
+        <v>1016</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2">
-        <v>200.5</v>
-      </c>
-      <c r="E2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2">
+        <v>-50.75</v>
+      </c>
+      <c r="D2" t="s">
         <v>11</v>
+      </c>
+      <c r="E2">
+        <v>2002</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3">
-        <v>102</v>
+        <v>9999</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3">
-        <v>350</v>
-      </c>
-      <c r="E3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3">
+        <v>936.61</v>
+      </c>
+      <c r="D3" t="s">
         <v>12</v>
+      </c>
+      <c r="E3">
+        <v>2002</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4">
-        <v>104</v>
+        <v>1013</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4">
-        <v>100.75</v>
-      </c>
-      <c r="E4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4">
+        <v>1052.43</v>
+      </c>
+      <c r="D4" t="s">
         <v>13</v>
+      </c>
+      <c r="E4">
+        <v>2001</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5">
-        <v>105</v>
-      </c>
-      <c r="C5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5">
-        <v>400</v>
-      </c>
-      <c r="E5" t="s">
+        <v>1004</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5">
+        <v>545.61</v>
+      </c>
+      <c r="D5" t="s">
         <v>14</v>
+      </c>
+      <c r="E5">
+        <v>2003</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6">
-        <v>102</v>
+        <v>1001</v>
       </c>
       <c r="B6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>645.39</v>
+      </c>
+      <c r="D6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>1020</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7">
+        <v>1839.25</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>1008</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8">
+        <v>1975.39</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>1003</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9">
+        <v>1505.52</v>
+      </c>
+      <c r="D9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>1011</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10">
+        <v>978.7</v>
+      </c>
+      <c r="D10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>1014</v>
+      </c>
+      <c r="B11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11">
+        <v>1768.6</v>
+      </c>
+      <c r="D11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>1014</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12">
+        <v>953.63</v>
+      </c>
+      <c r="D12" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>1019</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13">
+        <v>463.62</v>
+      </c>
+      <c r="D13" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>1016</v>
+      </c>
+      <c r="B14" t="s">
         <v>10</v>
       </c>
-      <c r="D6">
-        <v>350</v>
-      </c>
-      <c r="E6" t="s">
-        <v>12</v>
+      <c r="C14">
+        <v>142.36000000000001</v>
+      </c>
+      <c r="D14" t="s">
+        <v>23</v>
+      </c>
+      <c r="E14">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>1011</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15">
+        <v>1413.71</v>
+      </c>
+      <c r="D15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>1017</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16">
+        <v>101.95</v>
+      </c>
+      <c r="D16" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>1003</v>
+      </c>
+      <c r="B17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17">
+        <v>1410.63</v>
+      </c>
+      <c r="D17" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>1001</v>
+      </c>
+      <c r="B18" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18">
+        <v>1805.49</v>
+      </c>
+      <c r="D18" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>1006</v>
+      </c>
+      <c r="B19" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19">
+        <v>394.07</v>
+      </c>
+      <c r="D19" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>1014</v>
+      </c>
+      <c r="B20" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20">
+        <v>988.11</v>
+      </c>
+      <c r="D20" t="s">
+        <v>29</v>
+      </c>
+      <c r="E20">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>1003</v>
+      </c>
+      <c r="B21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21">
+        <v>1703.01</v>
+      </c>
+      <c r="D21" t="s">
+        <v>30</v>
+      </c>
+      <c r="E21">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>1019</v>
+      </c>
+      <c r="B22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22">
+        <v>1760.59</v>
+      </c>
+      <c r="D22" t="s">
+        <v>31</v>
+      </c>
+      <c r="E22">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>1016</v>
+      </c>
+      <c r="B23" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23">
+        <v>1606.09</v>
+      </c>
+      <c r="D23" t="s">
+        <v>32</v>
+      </c>
+      <c r="E23">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>1017</v>
+      </c>
+      <c r="B24" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24">
+        <v>1995.53</v>
+      </c>
+      <c r="D24" t="s">
+        <v>33</v>
+      </c>
+      <c r="E24">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>1002</v>
+      </c>
+      <c r="B25" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25">
+        <v>1161.67</v>
+      </c>
+      <c r="D25" t="s">
+        <v>34</v>
+      </c>
+      <c r="E25">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>1008</v>
+      </c>
+      <c r="B26" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26">
+        <v>819.26</v>
+      </c>
+      <c r="D26" t="s">
+        <v>35</v>
+      </c>
+      <c r="E26">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>1005</v>
+      </c>
+      <c r="B27" t="s">
+        <v>10</v>
+      </c>
+      <c r="C27">
+        <v>1618.45</v>
+      </c>
+      <c r="D27" t="s">
+        <v>36</v>
+      </c>
+      <c r="E27">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>1019</v>
+      </c>
+      <c r="B28" t="s">
+        <v>5</v>
+      </c>
+      <c r="C28">
+        <v>1939.1</v>
+      </c>
+      <c r="D28" t="s">
+        <v>37</v>
+      </c>
+      <c r="E28">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>1018</v>
+      </c>
+      <c r="B29" t="s">
+        <v>5</v>
+      </c>
+      <c r="C29">
+        <v>616.79</v>
+      </c>
+      <c r="D29" t="s">
+        <v>38</v>
+      </c>
+      <c r="E29">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>1018</v>
+      </c>
+      <c r="B30" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30">
+        <v>1792.36</v>
+      </c>
+      <c r="D30" t="s">
+        <v>39</v>
+      </c>
+      <c r="E30">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>1015</v>
+      </c>
+      <c r="B31" t="s">
+        <v>8</v>
+      </c>
+      <c r="C31">
+        <v>1061.56</v>
+      </c>
+      <c r="D31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E31">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>1019</v>
+      </c>
+      <c r="B32" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32">
+        <v>449.51</v>
+      </c>
+      <c r="D32" t="s">
+        <v>41</v>
+      </c>
+      <c r="E32">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>1002</v>
+      </c>
+      <c r="B33" t="s">
+        <v>5</v>
+      </c>
+      <c r="C33">
+        <v>884.14</v>
+      </c>
+      <c r="D33" t="s">
+        <v>42</v>
+      </c>
+      <c r="E33">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>1009</v>
+      </c>
+      <c r="B34" t="s">
+        <v>10</v>
+      </c>
+      <c r="C34">
+        <v>1630.71</v>
+      </c>
+      <c r="D34" t="s">
+        <v>43</v>
+      </c>
+      <c r="E34">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>1010</v>
+      </c>
+      <c r="B35" t="s">
+        <v>8</v>
+      </c>
+      <c r="C35">
+        <v>1246.25</v>
+      </c>
+      <c r="D35" t="s">
+        <v>44</v>
+      </c>
+      <c r="E35">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>1017</v>
+      </c>
+      <c r="B36" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36">
+        <v>296.63</v>
+      </c>
+      <c r="D36" t="s">
+        <v>45</v>
+      </c>
+      <c r="E36">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>1011</v>
+      </c>
+      <c r="B37" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37">
+        <v>1019.97</v>
+      </c>
+      <c r="D37" t="s">
+        <v>46</v>
+      </c>
+      <c r="E37">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>1009</v>
+      </c>
+      <c r="B38" t="s">
+        <v>9</v>
+      </c>
+      <c r="C38">
+        <v>704.6</v>
+      </c>
+      <c r="D38" t="s">
+        <v>47</v>
+      </c>
+      <c r="E38">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A39">
+        <v>1017</v>
+      </c>
+      <c r="B39" t="s">
+        <v>8</v>
+      </c>
+      <c r="C39">
+        <v>457.83</v>
+      </c>
+      <c r="D39" t="s">
+        <v>48</v>
+      </c>
+      <c r="E39">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A40">
+        <v>1005</v>
+      </c>
+      <c r="B40" t="s">
+        <v>5</v>
+      </c>
+      <c r="C40">
+        <v>1279.83</v>
+      </c>
+      <c r="D40" t="s">
+        <v>49</v>
+      </c>
+      <c r="E40">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <v>1015</v>
+      </c>
+      <c r="B41" t="s">
+        <v>6</v>
+      </c>
+      <c r="C41">
+        <v>1544.84</v>
+      </c>
+      <c r="D41" t="s">
+        <v>50</v>
+      </c>
+      <c r="E41">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A42">
+        <v>1008</v>
+      </c>
+      <c r="B42" t="s">
+        <v>9</v>
+      </c>
+      <c r="C42">
+        <v>1871.14</v>
+      </c>
+      <c r="D42" t="s">
+        <v>51</v>
+      </c>
+      <c r="E42">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A43">
+        <v>1008</v>
+      </c>
+      <c r="B43" t="s">
+        <v>5</v>
+      </c>
+      <c r="C43">
+        <v>916.49</v>
+      </c>
+      <c r="D43" t="s">
+        <v>52</v>
+      </c>
+      <c r="E43">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A44">
+        <v>1010</v>
+      </c>
+      <c r="B44" t="s">
+        <v>9</v>
+      </c>
+      <c r="C44">
+        <v>1792.06</v>
+      </c>
+      <c r="D44" t="s">
+        <v>53</v>
+      </c>
+      <c r="E44">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>1009</v>
+      </c>
+      <c r="B45" t="s">
+        <v>5</v>
+      </c>
+      <c r="C45">
+        <v>733.04</v>
+      </c>
+      <c r="D45" t="s">
+        <v>54</v>
+      </c>
+      <c r="E45">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>1009</v>
+      </c>
+      <c r="B46" t="s">
+        <v>9</v>
+      </c>
+      <c r="C46">
+        <v>1843.31</v>
+      </c>
+      <c r="D46" t="s">
+        <v>55</v>
+      </c>
+      <c r="E46">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>1015</v>
+      </c>
+      <c r="B47" t="s">
+        <v>8</v>
+      </c>
+      <c r="C47">
+        <v>944.65</v>
+      </c>
+      <c r="D47" t="s">
+        <v>15</v>
+      </c>
+      <c r="E47">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A48">
+        <v>1004</v>
+      </c>
+      <c r="B48" t="s">
+        <v>8</v>
+      </c>
+      <c r="C48">
+        <v>406.47</v>
+      </c>
+      <c r="D48" t="s">
+        <v>56</v>
+      </c>
+      <c r="E48">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49">
+        <v>1003</v>
+      </c>
+      <c r="B49" t="s">
+        <v>6</v>
+      </c>
+      <c r="C49">
+        <v>1143.82</v>
+      </c>
+      <c r="D49" t="s">
+        <v>13</v>
+      </c>
+      <c r="E49">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A50">
+        <v>1011</v>
+      </c>
+      <c r="B50" t="s">
+        <v>8</v>
+      </c>
+      <c r="C50">
+        <v>1080.67</v>
+      </c>
+      <c r="D50" t="s">
+        <v>57</v>
+      </c>
+      <c r="E50">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A51">
+        <v>1001</v>
+      </c>
+      <c r="B51" t="s">
+        <v>6</v>
+      </c>
+      <c r="C51">
+        <v>111.56</v>
+      </c>
+      <c r="D51" t="s">
+        <v>58</v>
+      </c>
+      <c r="E51">
+        <v>2002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>